<commit_message>
Refactor PDF generation and update example data
Co-authored-by: selva <selva@uni-hildesheim.de>
</commit_message>
<xml_diff>
--- a/participants.xlsx
+++ b/participants.xlsx
@@ -448,34 +448,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Jane</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Doe</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>john.smith@email.com</t>
+          <t>jane.doe@email.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jane</t>
+          <t>John</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Doe</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>jane.johnson@email.com</t>
+          <t>john.doe@email.com</t>
         </is>
       </c>
     </row>

</xml_diff>